<commit_message>
Template unggah + perbaiki penjaga git di skrip push
</commit_message>
<xml_diff>
--- a/contoh/Template-01-Break-Deposito.xlsx
+++ b/contoh/Template-01-Break-Deposito.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -67,15 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -451,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -615,172 +607,164 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>wajib, 4-5 digit</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>angka</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>tanggal</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>tanggal</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>wajib, tanggal</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>jam hh:mm:ss</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>jam hh:mm:ss</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>teks, disamarkan</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>wajib, angka</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>angka</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>IDR / lainnya</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>angka desimal</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>teks, disamarkan</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr"/>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="Y2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
-        </is>
-      </c>
-      <c r="Z2" s="3" t="inlineStr">
-        <is>
-          <t>teks</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>01006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CAB.JAKARTA-GREEN GARDEN</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3450000000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>45520</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0.4000925925925926</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.4003472222222222</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>300010002826028</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>BUDI HARTONO</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>338944580.82</v>
+      </c>
+      <c r="M2" t="n">
+        <v>267178.08</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>209010000331601</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>BUDI HARTONO</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>MNC2413400</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PETUGAS CS CONTOH</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>MNC0410100</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>PENYELIA CONTOH</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>410100</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>TELLER CONTOH</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>410140</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>PENYELIA 2 CONTOH</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>01006</t>
+          <t>01001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAB.JAKARTA-GREEN GARDEN</t>
+          <t>CAB.JAKARTA-WISMA BUMIPUTERA</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3450000000</v>
+        <v>1200000000</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>45520</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>46250</v>
-      </c>
-      <c r="G3" s="4" t="n">
+      <c r="E3" s="3" t="n">
+        <v>45689</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>46237</v>
       </c>
-      <c r="H3" s="5" t="n">
-        <v>0.4000925925925926</v>
-      </c>
-      <c r="I3" s="5" t="n">
-        <v>0.4003472222222222</v>
+      <c r="H3" s="4" t="n">
+        <v>0.4270833333333333</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.4275694444444444</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>300010002826028</t>
+          <t>300010002826029</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>BUDI HARTONO</t>
+          <t>PT CONTOH SEJAHTERA</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>338944580.82</v>
+        <v>1200000000</v>
       </c>
       <c r="M3" t="n">
-        <v>267178.08</v>
+        <v>900000</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -788,7 +772,7 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>0.06</v>
+        <v>0.055</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -797,7 +781,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>BUDI HARTONO</t>
+          <t>PT CONTOH SEJAHTERA</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -807,7 +791,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>MNC2413400</t>
+          <t>MNC2413401</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -817,7 +801,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>MNC0410100</t>
+          <t>MNC0410101</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -827,7 +811,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>410100</t>
+          <t>410101</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -837,7 +821,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>410140</t>
+          <t>410141</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -849,50 +833,50 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01001</t>
+          <t>01008</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAB.JAKARTA-WISMA BUMIPUTERA</t>
+          <t>CAB.JAKARTA-PURI INDAH</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1200000000</v>
+        <v>500000000</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>45689</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>46254</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>46237</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>0.4275694444444444</v>
+      <c r="E4" s="3" t="n">
+        <v>46034</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.584849537037037</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.5854166666666667</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>300010002826029</t>
+          <t>300010002826030</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>PT CONTOH SEJAHTERA</t>
+          <t>SITI RAHAYU</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1200000000</v>
+        <v>500000000</v>
       </c>
       <c r="M4" t="n">
-        <v>900000</v>
+        <v>250000</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -900,7 +884,7 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>0.055</v>
+        <v>0.0575</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -909,7 +893,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PT CONTOH SEJAHTERA</t>
+          <t>SITI RAHAYU</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -919,7 +903,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>MNC2413401</t>
+          <t>MNC2413402</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -929,7 +913,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>MNC0410101</t>
+          <t>MNC0410102</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -939,7 +923,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>410101</t>
+          <t>410102</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -949,7 +933,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>410141</t>
+          <t>410142</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -961,50 +945,50 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>01008</t>
+          <t>01003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAB.JAKARTA-PURI INDAH</t>
+          <t>CAB.JAKARTA-WOLTER</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>500000000</v>
+        <v>750000000</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>46034</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>46277</v>
-      </c>
-      <c r="G5" s="4" t="n">
+      <c r="E5" s="3" t="n">
+        <v>45964</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>46329</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>46238</v>
       </c>
-      <c r="H5" s="5" t="n">
-        <v>0.584849537037037</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>0.5854166666666667</v>
+      <c r="H5" s="4" t="n">
+        <v>0.6945023148148148</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.6953703703703704</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>300010002826030</t>
+          <t>300010002826031</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>SITI RAHAYU</t>
+          <t>DEWI ANGGRAINI</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>500000000</v>
+        <v>748500000</v>
       </c>
       <c r="M5" t="n">
-        <v>250000</v>
+        <v>601500</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1012,7 +996,7 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>0.0575</v>
+        <v>0.0625</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1021,7 +1005,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>SITI RAHAYU</t>
+          <t>DEWI ANGGRAINI</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1031,7 +1015,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MNC2413402</t>
+          <t>MNC2413403</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -1041,7 +1025,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>MNC0410102</t>
+          <t>MNC0410103</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1051,7 +1035,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>410102</t>
+          <t>410103</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1061,7 +1045,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>410142</t>
+          <t>410143</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -1073,50 +1057,50 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01003</t>
+          <t>01004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAB.JAKARTA-WOLTER</t>
+          <t>CAB.JAKARTA-ROXY</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>750000000</v>
+        <v>250000000</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>45964</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>46329</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>46238</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>0.6945023148148148</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>0.6953703703703704</v>
+      <c r="E6" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.3373148148148148</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.3376157407407407</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>300010002826031</t>
+          <t>300010002826032</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>DEWI ANGGRAINI</t>
+          <t>CV MITRA CONTOH</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>748500000</v>
+        <v>250000000</v>
       </c>
       <c r="M6" t="n">
-        <v>601500</v>
+        <v>0</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1124,7 +1108,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>0.0625</v>
+        <v>0.05</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1133,7 +1117,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>DEWI ANGGRAINI</t>
+          <t>CV MITRA CONTOH</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1143,7 +1127,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>MNC2413403</t>
+          <t>MNC2413404</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1153,7 +1137,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>MNC0410103</t>
+          <t>MNC0410104</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1163,7 +1147,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>410103</t>
+          <t>410104</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1173,122 +1157,10 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>410143</t>
+          <t>410144</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
-        <is>
-          <t>PENYELIA 2 CONTOH</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>01004</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CAB.JAKARTA-ROXY</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>250000000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>46101</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>46239</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.3373148148148148</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>0.3376157407407407</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>300010002826032</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>CV MITRA CONTOH</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>250000000</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>IDR</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>209010000331601</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>CV MITRA CONTOH</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>MNC2413404</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>PETUGAS CS CONTOH</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>MNC0410104</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>PENYELIA CONTOH</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>410104</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>TELLER CONTOH</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>410144</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
         <is>
           <t>PENYELIA 2 CONTOH</t>
         </is>
@@ -1305,253 +1177,479 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>ATURAN YANG BERLAKU UNTUK KETIGA TEMPLATE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>1. Parser membaca sel berdasarkan POSISI kolom, bukan judulnya.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Judul boleh diganti bahasanya; URUTAN KOLOM TIDAK BOLEH BERUBAH.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Menyisipkan kolom di tengah menggeser semua kolom sesudahnya, dan</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   data akan masuk ke kolom yang salah TANPA pesan galat.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr"/>
+      <c r="A7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2. Kolom baru selalu ditambahkan di PALING KANAN, tidak pernah di tengah.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
+      <c r="A9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>3. Baris judul tidak boleh dipindah. Data dimulai pada baris yang sudah</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   ditentukan di tiap template (lihat catatan di lembar ini).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
+      <c r="A12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>4. Kode cabang harus sudah terdaftar di Master Cabang. Kalau belum,</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   seluruh barisnya ditolak dengan 'Kode cabang tidak dikenal'.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Unggah '01. Kode dan Nama Cabang.xlsx' lebih dulu di Langkah 0.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr"/>
+      <c r="A16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>5. Sel tanggal harus benar-benar bertipe TANGGAL di Excel, bukan teks.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Parser tidak menebak-nebak format; teks '01/08/2026' dibaca kosong.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr"/>
+      <c r="A19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>6. Kolom berlatar KUNING adalah tambahan Agustus 2026. Boleh dikosongkan;</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   berkas lama tanpa kolom itu tetap bisa diunggah.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Kolom berlatar ABU-ABU tidak dibaca parser - biarkan apa adanya.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr"/>
+      <c r="A23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>7. Unggah menghasilkan batch berstatus 'draft'. Data baru muncul di</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   dashboard setelah ditekan 'Komit' di tab Unggah.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr"/>
+      <c r="A26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>DAFTAR KOLOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Kolom Excel | indeks parser | judul | keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>------------------------------------------------------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   A  |  r[ 0]  |  Kode Cabang                      | wajib, 4-5 digit</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   B  |  r[ 1]  |  Nama Cabang (core)               | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   C  |  r[ 2]  |  Saldo                            | angka</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   D  |  r[ 3]  |  (tidak dibaca)                   | </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   E  |  r[ 4]  |  Tanggal Penempatan               | tanggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   F  |  r[ 5]  |  Tanggal Jatuh Tempo              | tanggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   G  |  r[ 6]  |  Tanggal Break                    | wajib, tanggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   H  |  r[ 7]  |  Waktu Awal                       | jam hh:mm:ss</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   I  |  r[ 8]  |  Waktu Akhir                      | jam hh:mm:ss</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   J  |  r[ 9]  |  Rekening Pendebetan              | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   K  |  r[10]  |  Nama Pemilik                     | teks, disamarkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   L  |  r[11]  |  Nominal                          | wajib, angka</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   M  |  r[12]  |  Penalti                          | angka</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   N  |  r[13]  |  Mata Uang                        | IDR / lainnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   O  |  r[14]  |  Rate                             | angka desimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   P  |  r[15]  |  Rekening Pencairan               | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Q  |  r[16]  |  Nama Pencairan                   | teks, disamarkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   R  |  r[17]  |  (tidak dibaca)                   | </t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   S  |  r[18]  |  CS ID                            | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   T  |  r[19]  |  CS Nama                          | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   U  |  r[20]  |  (tidak dibaca)                   | </t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   V  |  r[21]  |  FLM1 Nama                        | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   W  |  r[22]  |  Teller ID                        | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   X  |  r[23]  |  Teller Nama                      | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Y  |  r[24]  |  FLM2 ID                          | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Z  |  r[25]  |  FLM2 Nama                        | teks</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Kolom bertanda * adalah tambahan Agustus 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Kolom berjudul (tidak dibaca) memang dilewati parser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>KHUSUS BREAK DEPOSITO</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Nama lembar : Sheet1  (kalau berbeda, lembar PERTAMA yang dipakai)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>Baris judul : 1</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>Data mulai  : baris 2</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>Baris dilewati bila kolom A (Kode Cabang) kosong.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>Kolom wajib : Kode Cabang, Tanggal Break, Nominal.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>Kolom 4, 18 dan 21 tidak dibaca parser - di ekspor asli isinya</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>duplikat dari kolom lain.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>Kolom bebas berikutnya kalau perlu menambah field: kolom ke-27 (r[26]).</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
         <is>
           <t>Tanggal Break di luar rentang wajar TIDAK ditolak, hanya diberi</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
         <is>
           <t>peringatan. Batch 27 (Agustus 2026) lolos dengan seluruh tanggal</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>1984-05-24 karena itu - periksa hasil unggahan sebelum Komit.</t>
         </is>

</xml_diff>